<commit_message>
Anchor sourcing action timing to recorded commitment end
</commit_message>
<xml_diff>
--- a/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
+++ b/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra12902ed6cfd4f95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="Rb316df8b43614819"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="R3ea1ff2e299f4b4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="Rd93b1e25fcd6482e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Ra3f03fa6d2d34fc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="R79a7a88a61d44c79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R29804b8401ad49e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="Rcad4fbabf9954ec6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="Re9cc21951b004ea8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="R89ab7623f0af42bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R498e596ab1324581"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="R45852dbf61894d65"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -395,7 +395,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf1dd9d5263fd4daa"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R80a27eaae8734ef7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -882,7 +882,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b3552be735d4dcb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cadf48e348c433d"/>
 </x:worksheet>
 </file>
 
@@ -1300,7 +1300,7 @@
         <x:v>Strategic Sourcing</x:v>
       </x:c>
       <x:c r="F7" s="17" t="str">
-        <x:v>Draft carry-forward amendment before the Year 2 payment locks.</x:v>
+        <x:v>Draft carry-forward amendment before the 2026-10-14 Year 1 commitment anniversary.</x:v>
       </x:c>
       <x:c r="G7" s="17" t="str">
         <x:v>coverage:MER-TECH-DBX-001:2026-09;clause:MER-TECH-DBX-001:no_carry_forward;ap_recon:MER-TECH-DBX-001:2026-09</x:v>
@@ -1579,7 +1579,7 @@
         <x:v>Timing dependency</x:v>
       </x:c>
       <x:c r="B27" s="17" t="str">
-        <x:v>Resolve before year-end true-up and Year 2 payment authorization.</x:v>
+        <x:v>Resolve before 2026-10-14, when unused Year 1 commitment expires at the contract-year anniversary. Confirm any separate payment milestone with Finance.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Reject duplicate document IDs in package inventory
</commit_message>
<xml_diff>
--- a/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
+++ b/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R29804b8401ad49e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="Rcad4fbabf9954ec6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="Re9cc21951b004ea8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="R89ab7623f0af42bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R498e596ab1324581"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="R45852dbf61894d65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2b014623090d4cb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="R9b0a14416e9d44cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="Rca8598c95fcd45b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="R9b4a9432d9ba4841"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R9fed7e3407404682"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="Rb8053cb7deaa4446"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -395,7 +395,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R80a27eaae8734ef7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R38536fb0b70d4fb6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -882,7 +882,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cadf48e348c433d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcef1b12cb2114391"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Anchor sourcing action timing to recorded commitment end (#7755)
* Anchor sourcing action timing to recorded commitment end

* Reject duplicate document IDs in package inventory

---------

Co-authored-by: Anand Sundaram <anandsundaram-hash@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
+++ b/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra12902ed6cfd4f95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="Rb316df8b43614819"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="R3ea1ff2e299f4b4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="Rd93b1e25fcd6482e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Ra3f03fa6d2d34fc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="R79a7a88a61d44c79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2b014623090d4cb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="R9b0a14416e9d44cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="Rca8598c95fcd45b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="R9b4a9432d9ba4841"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R9fed7e3407404682"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="Rb8053cb7deaa4446"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -395,7 +395,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf1dd9d5263fd4daa"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R38536fb0b70d4fb6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -882,7 +882,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b3552be735d4dcb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcef1b12cb2114391"/>
 </x:worksheet>
 </file>
 
@@ -1300,7 +1300,7 @@
         <x:v>Strategic Sourcing</x:v>
       </x:c>
       <x:c r="F7" s="17" t="str">
-        <x:v>Draft carry-forward amendment before the Year 2 payment locks.</x:v>
+        <x:v>Draft carry-forward amendment before the 2026-10-14 Year 1 commitment anniversary.</x:v>
       </x:c>
       <x:c r="G7" s="17" t="str">
         <x:v>coverage:MER-TECH-DBX-001:2026-09;clause:MER-TECH-DBX-001:no_carry_forward;ap_recon:MER-TECH-DBX-001:2026-09</x:v>
@@ -1579,7 +1579,7 @@
         <x:v>Timing dependency</x:v>
       </x:c>
       <x:c r="B27" s="17" t="str">
-        <x:v>Resolve before year-end true-up and Year 2 payment authorization.</x:v>
+        <x:v>Resolve before 2026-10-14, when unused Year 1 commitment expires at the contract-year anniversary. Confirm any separate payment milestone with Finance.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">

</xml_diff>